<commit_message>
Add annual hours and a separate insurance census template
</commit_message>
<xml_diff>
--- a/site/ThousandSquared_Data_Template.xlsx
+++ b/site/ThousandSquared_Data_Template.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Employees" sheetId="1" r:id="Rc99322fed65940ed"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly Hours" sheetId="2" r:id="R47c43d543c234792"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Employee Coverage" sheetId="3" r:id="Rc95433b58d784913"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Covered Family" sheetId="4" r:id="R7c42beed78304e0e"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="5" r:id="R38d42ccbf04048d3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Employees" sheetId="1" r:id="R42477210eb8d42d9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly Hours" sheetId="2" r:id="R6be8471da31f4e91"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Insurance Census" sheetId="3" r:id="R044a0533289a4b33"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Covered Family" sheetId="4" r:id="R9c3b8663ddfb4caf"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="5" r:id="Rb320a2401031481a"/>
   </sheets>
 </workbook>
 </file>
@@ -484,6 +484,7 @@
     <col min="13" max="13" width="13" hidden="0" customWidth="1"/>
     <col min="14" max="14" width="13" hidden="0" customWidth="1"/>
     <col min="15" max="15" width="13" hidden="0" customWidth="1"/>
+    <col min="16" max="16" width="20" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="42" customHeight="1">
@@ -532,6 +533,9 @@
       <c r="O1" s="6" t="str">
         <v>Hours Dec</v>
       </c>
+      <c r="P1" s="6" t="str">
+        <v>Hours Total</v>
+      </c>
     </row>
     <row r="2" ht="25" customHeight="1">
       <c r="A2" s="10" t="str">
@@ -578,6 +582,9 @@
       </c>
       <c r="O2" s="16" t="n">
         <v>160</v>
+      </c>
+      <c r="P2" s="11" t="n">
+        <v>1920</v>
       </c>
     </row>
   </sheetData>
@@ -809,138 +816,146 @@
     </row>
     <row r="6" ht="48" customHeight="1">
       <c r="A6" s="21" t="str">
-        <v>Monthly hours</v>
+        <v>Hours or FT/PT status</v>
       </c>
       <c r="B6" s="22" t="str">
-        <v>Recommended for monthly ACA status: hours of service, including paid non-work time. Use 0 for a true zero and leave unknown values blank.</v>
+        <v>Use Hours Jan through Hours Dec for monthly hours, Hours Total for annual hours, or FT PT Status on Employees for an employer-provided FT/PT classification. Supply the applicable option; all three are not required.</v>
       </c>
       <c r="C6" s="1"/>
     </row>
     <row r="7" ht="48" customHeight="1">
       <c r="A7" s="21" t="str">
-        <v>Identifiers</v>
+        <v>Monthly hours</v>
       </c>
       <c r="B7" s="22" t="str">
-        <v>Use the same employee SSN across tabs. Employee ID is helpful for matching but does not replace the employee SSN needed for generation. Keep SSNs and ZIPs as text.</v>
+        <v>Include paid hours of service, including paid non-work time. Use 0 for a true zero and leave unknown values blank. Monthly hours are preferred when status changes.</v>
       </c>
       <c r="C7" s="1"/>
     </row>
     <row r="8" ht="48" customHeight="1">
       <c r="A8" s="21" t="str">
-        <v>Birth and termination dates</v>
+        <v>Identifiers</v>
       </c>
       <c r="B8" s="22" t="str">
-        <v>Employee DOB is needed for ICHRA age-based pricing and where covered-person identification requires it. Supply termination dates when applicable.</v>
+        <v>Use the same employee SSN across tabs. Employee ID is helpful for matching but does not replace the employee SSN needed for generation. Keep SSNs and ZIPs as text.</v>
       </c>
       <c r="C8" s="1"/>
     </row>
     <row r="9" ht="48" customHeight="1">
       <c r="A9" s="21" t="str">
-        <v>Coverage</v>
+        <v>Birth and termination dates</v>
       </c>
       <c r="B9" s="22" t="str">
-        <v>Use actual coverage dates. Leave Coverage Term Date blank for ongoing coverage. Add a separate row for each period; repeated employee SSNs are expected here.</v>
+        <v>Employee DOB is needed for ICHRA age-based pricing and where covered-person identification requires it. Supply termination dates when applicable.</v>
       </c>
       <c r="C9" s="1"/>
     </row>
     <row r="10" ht="48" customHeight="1">
       <c r="A10" s="21" t="str">
-        <v>Covered family</v>
+        <v>Insurance Census</v>
       </c>
       <c r="B10" s="22" t="str">
-        <v>For applicable self-insured/ICHRA reporting: one row per covered family member and period. Subscriber SSN identifies the employee; SSN identifies that family member.</v>
+        <v>The insurance template is the Insurance Census tab. Use actual coverage dates. Leave Coverage Term Date blank for ongoing coverage. Add a separate row for each period; repeated employee SSNs are expected here.</v>
       </c>
       <c r="C10" s="1"/>
     </row>
     <row r="11" ht="48" customHeight="1">
       <c r="A11" s="21" t="str">
-        <v>Family identification</v>
+        <v>Covered family</v>
       </c>
       <c r="B11" s="22" t="str">
-        <v>Provide each covered person’s name and SSN. If SSN is unavailable, provide DOB and review the applicable identification requirements. Include actual coverage dates.</v>
+        <v>For applicable self-insured/ICHRA reporting: one row per covered family member and period. Subscriber SSN identifies the employee; SSN identifies that family member.</v>
       </c>
       <c r="C11" s="1"/>
     </row>
     <row r="12" ht="48" customHeight="1">
       <c r="A12" s="21" t="str">
-        <v>Classes and locations</v>
+        <v>Family identification</v>
       </c>
       <c r="B12" s="22" t="str">
-        <v>Helpful when policies vary: employee class, work location, ACA full-time status and county. Class and location names should match company setup.</v>
+        <v>Provide each covered person’s name and SSN. If SSN is unavailable, provide DOB and review the applicable identification requirements. Include actual coverage dates.</v>
       </c>
       <c r="C12" s="1"/>
     </row>
     <row r="13" ht="48" customHeight="1">
       <c r="A13" s="21" t="str">
-        <v>Special situations</v>
+        <v>Classes and locations</v>
       </c>
       <c r="B13" s="22" t="str">
-        <v>Supply COBRA, union, leave and stability-period facts and dates where applicable; review these in the application rather than assuming one flag covers every case.</v>
+        <v>Helpful when policies vary: employee class, work location, ACA full-time status and county. Class and location names should match company setup.</v>
       </c>
       <c r="C13" s="1"/>
     </row>
     <row r="14" ht="48" customHeight="1">
       <c r="A14" s="21" t="str">
-        <v>ICHRA</v>
+        <v>Special situations</v>
       </c>
       <c r="B14" s="22" t="str">
-        <v>Complete allowance, ZIP basis and plan-year settings in the questionnaire. Supply employee DOB, applicable residence/work location and county when required.</v>
+        <v>Supply COBRA, union, leave and stability-period facts and dates where applicable; review these in the application rather than assuming one flag covers every case.</v>
       </c>
       <c r="C14" s="1"/>
     </row>
     <row r="15" ht="48" customHeight="1">
       <c r="A15" s="21" t="str">
-        <v>Company questionnaire</v>
+        <v>ICHRA</v>
       </c>
       <c r="B15" s="22" t="str">
-        <v>Enter legal name, EIN, address, reporting year, plan type, offer scope, minimum value/MEC, waiting policy, contribution amounts and safe harbor there.</v>
+        <v>Complete allowance, ZIP basis and plan-year settings in the questionnaire. Supply employee DOB, applicable residence/work location and county when required.</v>
       </c>
       <c r="C15" s="1"/>
     </row>
     <row r="16" ht="48" customHeight="1">
       <c r="A16" s="21" t="str">
-        <v>Annual totals</v>
+        <v>Company questionnaire</v>
       </c>
       <c r="B16" s="22" t="str">
-        <v>Monthly hours are preferred. An annual total alone does not identify hours in hire/termination months or prove original cumulative-hours eligibility.</v>
+        <v>Enter legal name, EIN, address, reporting year, plan type, offer scope, minimum value/MEC, waiting policy, contribution amounts and safe harbor there.</v>
       </c>
       <c r="C16" s="1"/>
     </row>
     <row r="17" ht="48" customHeight="1">
       <c r="A17" s="21" t="str">
-        <v>Existing reports</v>
+        <v>Annual totals</v>
       </c>
       <c r="B17" s="22" t="str">
-        <v>This format is optional. Existing payroll and insurer spreadsheets can also be mapped. Review diagnostics and correct missing facts before generating or filing.</v>
+        <v>Hours Total is the annual hours input, not an extra month. The example 1,920 matches twelve months of 160. If using annual hours only, clear the fictional monthly hours; annual totals do not describe month-to-month status changes.</v>
       </c>
       <c r="C17" s="1"/>
     </row>
     <row r="18" ht="48" customHeight="1">
       <c r="A18" s="21" t="str">
-        <v>Dates and privacy</v>
+        <v>FT/PT classification</v>
       </c>
       <c r="B18" s="22" t="str">
-        <v>Use real Excel dates displayed as YYYY-MM-DD. Upload completed files through the application, not a public contact form or inquiry email.</v>
+        <v>Use FT or PT in Employees: FT PT Status. This imported indicator is one employee-level value, not twelve monthly status fields. Review changes in monthly status in the application.</v>
       </c>
       <c r="C18" s="1"/>
     </row>
     <row r="19" ht="48" customHeight="1">
       <c r="A19" s="21" t="str">
+        <v>Existing reports</v>
+      </c>
+      <c r="B19" s="22" t="str">
+        <v>This format is optional. Existing payroll and insurer spreadsheets can also be mapped. Review diagnostics and correct missing facts before generating or filing.</v>
+      </c>
+      <c r="C19" s="1"/>
+    </row>
+    <row r="20" ht="48" customHeight="1">
+      <c r="A20" s="21" t="str">
+        <v>Dates and privacy</v>
+      </c>
+      <c r="B20" s="22" t="str">
+        <v>Use real Excel dates displayed as YYYY-MM-DD. Upload completed files through the application, not a public contact form or inquiry email.</v>
+      </c>
+      <c r="C20" s="1"/>
+    </row>
+    <row r="21" ht="48" customHeight="1">
+      <c r="A21" s="21" t="str">
         <v>Example year</v>
       </c>
-      <c r="B19" s="22" t="str">
+      <c r="B21" s="22" t="str">
         <v>2025 is illustrative only. Replace the sample dates and year with the reporting period you are preparing.</v>
       </c>
-      <c r="C19" s="1"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="1"/>
-      <c r="B20" s="1"/>
-      <c r="C20" s="1"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="1"/>
-      <c r="B21" s="1"/>
       <c r="C21" s="1"/>
     </row>
     <row r="22">

</xml_diff>